<commit_message>
SEO prune agressif: noindex cryptos + fiches cartes non evaluees + duplicatas be/at (concentration qualite)
</commit_message>
<xml_diff>
--- a/seo/backlinks-outreach.xlsx
+++ b/seo/backlinks-outreach.xlsx
@@ -8,18 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plateformes journalistes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annuaires surs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journalistes FR" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journalistes EN-Intl" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journalistes DE-ES-IT" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails prêts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plateformes journalistes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annuaires surs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journalistes FR" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journalistes EN-Intl" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journalistes DE-ES-IT" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plateformes journalistes'!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Annuaires surs'!$A$1:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Journalistes FR'!$A$1:$K$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Journalistes EN-Intl'!$A$1:$K$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Journalistes DE-ES-IT'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Plateformes journalistes'!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Annuaires surs'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Journalistes FR'!$A$1:$K$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Journalistes EN-Intl'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Journalistes DE-ES-IT'!$A$1:$K$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +59,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +84,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
   </fills>
@@ -108,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -131,6 +141,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -591,7 +608,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>1) Page « Contact / Proposer un sujet » du média.  2) X / LinkedIn du journaliste.  3) Pattern prenom.nom@media.xx (à vérifier).</t>
+          <t>1) Page « Contact / Proposer un sujet » du média.  2) Page auteur / byline du journaliste sur le site du média.  3) Pattern d'email prenom@media.xx ou prenom.nom@media.xx (à vérifier).</t>
         </is>
       </c>
     </row>
@@ -625,6 +642,440 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="95" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Réf</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Marché</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Cible</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Objet</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Corps de l'email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="170" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>The Big Whale — Grégory Raymond</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Exclu pour The Big Whale : les cartes crypto versent 34 % du cashback promis</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Grégory,
+Vous avez bâti The Big Whale sur l'indépendance vis-à-vis des promesses du secteur. J'ai des données qui en démontent une, le cashback des cartes crypto.
+On a analysé 95 cartes disponibles en Europe. Cashback affiché moyen : 4,29 %. Cashback réel sans staking : 1,07 %. Carte par carte, seuls 34 % du cashback affiché sont réellement versés. Une carte sur deux affiche 0 % de cashback de base. Championne de l'écart, Bleap, 20 % annoncés pour 1 % réel.
+Tout est vérifié à la main, disponible par pays, méthodologie ouverte. Je vous propose l'exclu 48 h avant les autres rédactions.
+L'étude : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="170" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>FR-gén</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Générique FR (aucun média cité)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="170" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Journal du Coin — Magali Bourdou</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback surgonflé des cartes crypto</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Le Journal du Coin alerte souvent sur les pièges du secteur. En voici un, chiffré.
+On a passé au crible 95 cartes crypto en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % promis en moyenne, 1,07 % réel. La moitié des cartes affichent 0 % de base. Le pire écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Données vérifiées à la main, par pays, méthodologie transparente : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux vous préparer le détail carte par carte ou un jeu de chiffres exclusif pour un papier.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="170" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Cryptoast — Clément Wardzala</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Analyse chiffrée sur 95 cartes crypto, méthodologie ouverte</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Clément,
+Cryptoast publie des analyses documentées et vérifiables. J'ai une étude taillée pour ce format.
+95 cartes crypto analysées en Europe, une seule question : combien de cashback est réellement versé par rapport à l'affiche. Réponse, 34 %. Le détail : 4,29 % promis en moyenne, 1,07 % touché sans staking, une carte sur deux à 0 % de base.
+La méthodologie est publiée sur la page, chaque chiffre est traçable : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je fournis volontiers les données brutes par carte et par marché si vous voulez creuser un angle.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="170" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>BFM Business — Antoine Larigaudrie</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Sujet chronique : on vous promet 10 % de cashback, vous touchez 2 %</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Antoine,
+Un sujet taillé pour une chronique conso de deux minutes.
+Les cartes crypto affichent des cashbacks à deux chiffres. Sur 95 cartes analysées en Europe, le taux réellement versé sans staking tombe à 34 % de la promesse. Exemple parlant, Bleap annonce 20 % et en verse 1 %. Une carte sur deux ne donne aucun cashback de base.
+Les chiffres et la méthode sont ici : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux passer en plateau ou fournir un commentaire chiffré quand vous voulez.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="170" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>CoinDesk — Francisco Rodrigues</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Data for your crypto-card coverage: advertised vs real cashback</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Hello Francisco,
+Your piece on crypto card spending passing $1 billion caught my eye, the Kraken Krak Card numbers in particular. I have a dataset that fits the same beat from the consumer side.
+We analysed 95 crypto cards in Europe. Advertised cashback averages 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. Bleap advertises 20% and pays 1%.
+Hand-checked, broken down by country, open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card data or a quote on how the advertised-versus-real gap looks across issuers.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="170" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>5b</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>CoinDesk — JP Koning</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Stablecoin cards: what the advertised cashback actually pays out</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Hello JP,
+You cover the mechanics of stablecoins and payments more closely than most. One under-reported piece of card economics: the cashback that sells the card rarely lands.
+Across 95 European crypto cards, advertised cashback averages 4.29% but the real rate without staking is 1.07%. Half pay zero base cashback. The gap looks structural, not incidental.
+Data and methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Glad to share the raw numbers for a payments-economics angle.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="170" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Générique EN</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="170" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>BTC-ECHO — Sven Wagenknecht</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Datenstudie: Krypto-Karten zahlen nur 34 % des versprochenen Cashbacks</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Hallo Herr Wagenknecht,
+ein Verbraucherthema mit eigenen Daten.
+Wir haben 93 in Europa verfügbare Krypto-Karten ausgewertet. Der beworbene Cashback liegt im Schnitt bei 4,29 %. Real, ohne Staking, sind es 1,07 %. Pro Karte werden im Schnitt nur 34 % des beworbenen Cashbacks gezahlt. Jede zweite Karte zahlt gar keinen Basis-Cashback. Der größte Abstand: Bleap, 20 % beworben, 1 % real.
+Alle Zahlen sind handgeprüft, nach Land aufgeschlüsselt, mit offener Methodik: https://topcryptocards.eu/etudes/krypto-karten-2026
+Gern liefere ich die vollständigen Daten pro Karte, Zahlen für den DACH-Raum oder ein Zitat.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="170" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Générique ES</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Estudio con datos: las tarjetas cripto pagan solo el 34 % del cashback que prometen</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Hola,
+Un ángulo de consumo con datos propios.
+Hemos analizado 95 tarjetas cripto disponibles en Europa. El cashback anunciado es del 4,29 % de media. El real, sin staking, baja al 1,07 %. Por tarjeta, de media solo se paga el 34 % del cashback anunciado. Una de cada dos tarjetas no da cashback base. La mayor diferencia es Bleap, 20 % anunciado frente a 1 % real.
+Cada cifra está verificada a mano, desglosada por país y con metodología abierta: https://topcryptocards.eu/etudes/tarjetas-cripto-2026
+Puedo facilitar los datos completos por tarjeta, cifras del mercado español o una cita.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="170" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Générique IT</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Studio con dati: le carte crypto pagano solo il 34 % del cashback promesso</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Salve,
+Un taglio consumer con dati originali.
+Abbiamo analizzato 95 carte crypto disponibili in Europa. Il cashback pubblicizzato è in media del 4,29 %. Quello reale, senza staking, scende allo 1,07 %. Per carta, in media viene versato solo il 34 % del cashback pubblicizzato. Una carta su due non dà alcun cashback base. Il divario più ampio è Bleap, 20 % pubblicizzato contro 1 % reale.
+Ogni dato è verificato a mano, suddiviso per paese, con metodologia aperta: https://topcryptocards.eu/etudes/carte-crypto-2026
+Posso fornire i dati completi per carta, i numeri del mercato italiano o una dichiarazione.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="170" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Générique PT</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Estudo com dados: os cartões crypto pagam só 34 % do cashback que prometem</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Olá,
+Um ângulo de consumo com dados próprios, e um lado fiscal que interessa em Portugal.
+Analisámos 95 cartões crypto disponíveis na Europa. O cashback anunciado é em média de 4,29 %. O real, sem staking, cai para 1,07 %. Por cartão, em média só é pago 34 % do cashback anunciado. Um em cada dois cartões não dá cashback de base. A maior diferença é da Bleap, 20 % anunciado contra 1 % real.
+Detalhe importante para o leitor português: pagar diretamente com cripto conta como alienação e pode gerar mais-valia tributável (28 % se detida há menos de um ano). Recebê-lo em token adiciona ainda risco de volatilidade.
+Cada número está verificado à mão, por país, com metodologia aberta: https://topcryptocards.eu/etudes/cartoes-crypto-2026
+Posso fornecer os dados completos por cartão, números do mercado português ou uma citação.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1018,7 +1469,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1265,13 +1716,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1285,6 +1736,8 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="85" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1343,6 +1796,16 @@
           <t>Lien obtenu</t>
         </is>
       </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>Objet email</t>
+        </is>
+      </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>Corps email (à copier)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -1372,7 +1835,7 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>X @gregory_raymond · thebigwhale.io · LinkedIn</t>
+          <t>contact@thebigwhale.io · graymond@thebigwhale.io (à confirmer, format initiale+nom)</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -1388,6 +1851,22 @@
       <c r="I2" s="7" t="inlineStr"/>
       <c r="J2" s="6" t="inlineStr"/>
       <c r="K2" s="7" t="inlineStr"/>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>Exclu pour The Big Whale : les cartes crypto versent 34 % du cashback promis</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Grégory,
+Vous avez bâti The Big Whale sur l'indépendance vis-à-vis des promesses du secteur. J'ai des données qui en démontent une, le cashback des cartes crypto.
+On a analysé 95 cartes disponibles en Europe. Cashback affiché moyen : 4,29 %. Cashback réel sans staking : 1,07 %. Carte par carte, seuls 34 % du cashback affiché sont réellement versés. Une carte sur deux affiche 0 % de cashback de base. Championne de l'écart, Bleap, 20 % annoncés pour 1 % réel.
+Tout est vérifié à la main, disponible par pays, méthodologie ouverte. Je vous propose l'exclu 48 h avant les autres rédactions.
+L'étude : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1417,7 +1896,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>LinkedIn (Raphaël Bloch)</t>
+          <t>rbloch@thebigwhale.io</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -1433,6 +1912,22 @@
       <c r="I3" s="7" t="inlineStr"/>
       <c r="J3" s="6" t="inlineStr"/>
       <c r="K3" s="7" t="inlineStr"/>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>Exclu pour The Big Whale : les cartes crypto versent 34 % du cashback promis</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Raphaël,
+Vous avez bâti The Big Whale sur l'indépendance vis-à-vis des promesses du secteur. J'ai des données qui en démontent une, le cashback des cartes crypto.
+On a analysé 95 cartes disponibles en Europe. Cashback affiché moyen : 4,29 %. Cashback réel sans staking : 1,07 %. Carte par carte, seuls 34 % du cashback affiché sont réellement versés. Une carte sur deux affiche 0 % de cashback de base. Championne de l'écart, Bleap, 20 % annoncés pour 1 % réel.
+Tout est vérifié à la main, disponible par pays, méthodologie ouverte. Je vous propose l'exclu 48 h avant les autres rédactions.
+L'étude : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1447,12 +1942,12 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Rémy Rosciano (+ frères Ermisse)</t>
+          <t>Magali Bourdou</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Fondateurs</t>
+          <t>Rédactrice en chef</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -1462,7 +1957,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>journalducoin.com (proposer un sujet) · X @LeJournalDuCoin</t>
+          <t>journalducoin.com/lequipe (icône email à cliquer) · magali@journalducoin.com (à confirmer) · éviter le formulaire commercial</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1478,6 +1973,21 @@
       <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="7" t="inlineStr"/>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback surgonflé des cartes crypto</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Magali,
+Le Journal du Coin alerte souvent sur les pièges du secteur. En voici un, chiffré.
+On a passé au crible 95 cartes crypto en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % promis en moyenne, 1,07 % réel. La moitié des cartes affichent 0 % de base. Le pire écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Données vérifiées à la main, par pays, méthodologie transparente : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux vous préparer le détail carte par carte ou un jeu de chiffres exclusif pour un papier.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1492,12 +2002,12 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Maximilien Prué</t>
+          <t>Clément Wardzala</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Rédacteur en chef</t>
+          <t>Directeur de la publication</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1507,7 +2017,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>cryptoast.fr/team + page contact · LinkedIn</t>
+          <t>cryptoast.fr/author/clement · kit presse cryptoast.fr/presskit · clement@cryptoast.fr (à confirmer)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1523,6 +2033,21 @@
       <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Analyse chiffrée sur 95 cartes crypto, méthodologie ouverte</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Clément,
+Cryptoast publie des analyses documentées et vérifiables. J'ai une étude taillée pour ce format.
+95 cartes crypto analysées en Europe, une seule question : combien de cashback est réellement versé par rapport à l'affiche. Réponse, 34 %. Le détail : 4,29 % promis en moyenne, 1,07 % touché sans staking, une carte sur deux à 0 % de base.
+La méthodologie est publiée sur la page, chaque chiffre est traçable : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je fournis volontiers les données brutes par carte et par marché si vous voulez creuser un angle.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -1552,7 +2077,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>LinkedIn (Vincent Maire)</t>
+          <t>cryptoast.fr/author/vincent-maire · vincent@cryptoast.fr (à confirmer)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1568,6 +2093,21 @@
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="7" t="inlineStr"/>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Analyse chiffrée sur 95 cartes crypto, méthodologie ouverte</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Vincent,
+Cryptoast publie des analyses documentées et vérifiables. J'ai une étude taillée pour ce format.
+95 cartes crypto analysées en Europe, une seule question : combien de cashback est réellement versé par rapport à l'affiche. Réponse, 34 %. Le détail : 4,29 % promis en moyenne, 1,07 % touché sans staking, une carte sur deux à 0 % de base.
+La méthodologie est publiée sur la page, chaque chiffre est traçable : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je fournis volontiers les données brutes par carte et par marché si vous voulez creuser un angle.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1597,7 +2137,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>cointribune.com contact · X @Cointribune</t>
+          <t>cointribune.com (page contact rédaction)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1613,6 +2153,21 @@
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -1642,7 +2197,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>coinacademy.fr contact · X @CoinAcademy_</t>
+          <t>coinacademy.fr (page contact)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1658,6 +2213,21 @@
       <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1687,7 +2257,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>BFM Business (contact rédaction) · X</t>
+          <t>bfmbusiness.com (contact rédaction crypto)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1703,6 +2273,21 @@
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Sujet chronique : on vous promet 10 % de cashback, vous touchez 2 %</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour Antoine,
+Un sujet taillé pour une chronique conso de deux minutes.
+Les cartes crypto affichent des cashbacks à deux chiffres. Sur 95 cartes analysées en Europe, le taux réellement versé sans staking tombe à 34 % de la promesse. Exemple parlant, Bleap annonce 20 % et en verse 1 %. Une carte sur deux ne donne aucun cashback de base.
+Les chiffres et la méthode sont ici : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux passer en plateau ou fournir un commentaire chiffré quand vous voulez.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -1732,7 +2317,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>LinkedIn (Gilles Quoistiaux)</t>
+          <t>page contact rédaction éco de son média</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1748,6 +2333,21 @@
       <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr"/>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1793,6 +2393,21 @@
       <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="6" t="inlineStr"/>
       <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1838,6 +2453,21 @@
       <c r="I12" s="7" t="inlineStr"/>
       <c r="J12" s="6" t="inlineStr"/>
       <c r="K12" s="7" t="inlineStr"/>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -1867,7 +2497,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Repérer via articles récents + LinkedIn</t>
+          <t>lesechos.fr (contact rédaction) · repérer la byline crypto récente</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1883,6 +2513,21 @@
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="6" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1928,6 +2573,21 @@
       <c r="I14" s="7" t="inlineStr"/>
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="7" t="inlineStr"/>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1973,6 +2633,21 @@
       <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="6" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>Données maison : le cashback réel des cartes crypto (étude sur 95 cartes)</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>Bonjour,
+Un angle conso appuyé par des données maison.
+On a passé au crible 95 cartes crypto disponibles en Europe. Le cashback réellement versé sans staking n'atteint que 34 % de ce qui est affiché : 4,29 % annoncés en moyenne, 1,07 % réellement touchés. Une carte sur deux affiche 0 % de cashback de base. Le plus gros écart revient à Bleap, 20 % annoncés pour 1 % réel.
+Chaque chiffre est vérifié à la main, décliné par pays, méthodologie ouverte : https://topcryptocards.eu/etudes/cartes-crypto-2026
+Je peux fournir le détail carte par carte, les chiffres par marché, ou un commentaire à citer.
+Thomas, TopCryptoCards, comparateur indépendant de cartes crypto en Europe</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K15"/>
@@ -1985,13 +2660,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2005,6 +2680,8 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="85" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2063,6 +2740,16 @@
           <t>Lien obtenu</t>
         </is>
       </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>Objet email</t>
+        </is>
+      </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>Corps email (à copier)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -2108,6 +2795,21 @@
       <c r="I2" s="7" t="inlineStr"/>
       <c r="J2" s="6" t="inlineStr"/>
       <c r="K2" s="7" t="inlineStr"/>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -2153,6 +2855,21 @@
       <c r="I3" s="7" t="inlineStr"/>
       <c r="J3" s="6" t="inlineStr"/>
       <c r="K3" s="7" t="inlineStr"/>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -2198,6 +2915,21 @@
       <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="7" t="inlineStr"/>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2243,6 +2975,21 @@
       <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2288,6 +3035,21 @@
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="7" t="inlineStr"/>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2333,6 +3095,21 @@
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2378,6 +3155,21 @@
       <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2423,6 +3215,21 @@
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -2468,6 +3275,21 @@
       <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr"/>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -2513,6 +3335,21 @@
       <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="6" t="inlineStr"/>
       <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Data study: crypto cards pay just 34% of the cashback they advertise</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Hello,
+A consumer angle backed by original data.
+We analysed 95 crypto cards available across Europe. Average advertised cashback is 4.29%. The real rate without staking is 1.07%. Per card, only 34% of the advertised cashback actually lands. One card in two pays zero base cashback. The widest gap is Bleap, 20% advertised against 1% real.
+Every figure is hand-checked, broken down by country, with an open methodology: https://topcryptocards.eu/etudes/crypto-cards-2026
+Happy to share the full per-card dataset, market-level numbers, or a quote.
+Thomas, TopCryptoCards, independent crypto card comparison in Europe</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K11"/>
@@ -2525,13 +3362,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2545,6 +3382,8 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="85" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2603,6 +3442,16 @@
           <t>Lien obtenu</t>
         </is>
       </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>Objet email</t>
+        </is>
+      </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>Corps email (à copier)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -2632,7 +3481,7 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>btc-echo.de (Redaktion) · LinkedIn</t>
+          <t>btc-echo.de (Redaktion)</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -2648,6 +3497,21 @@
       <c r="I2" s="7" t="inlineStr"/>
       <c r="J2" s="6" t="inlineStr"/>
       <c r="K2" s="7" t="inlineStr"/>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>Datenstudie: Krypto-Karten zahlen nur 34 % des versprochenen Cashbacks</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>Hallo Herr Wagenknecht,
+ein Verbraucherthema mit eigenen Daten.
+Wir haben 93 in Europa verfügbare Krypto-Karten ausgewertet. Der beworbene Cashback liegt im Schnitt bei 4,29 %. Real, ohne Staking, sind es 1,07 %. Pro Karte werden im Schnitt nur 34 % des beworbenen Cashbacks gezahlt. Jede zweite Karte zahlt gar keinen Basis-Cashback. Der größte Abstand: Bleap, 20 % beworben, 1 % real.
+Alle Zahlen sind handgeprüft, nach Land aufgeschlüsselt, mit offener Methodik: https://topcryptocards.eu/etudes/krypto-karten-2026
+Gern liefere ich die vollständigen Daten pro Karte, Zahlen für den DACH-Raum oder ein Zitat.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -2693,6 +3557,21 @@
       <c r="I3" s="7" t="inlineStr"/>
       <c r="J3" s="6" t="inlineStr"/>
       <c r="K3" s="7" t="inlineStr"/>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>Datenstudie: Krypto-Karten zahlen nur 34 % des versprochenen Cashbacks</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>Hallo Redaktion,
+ein Verbraucherthema mit eigenen Daten.
+Wir haben 93 in Europa verfügbare Krypto-Karten ausgewertet. Der beworbene Cashback liegt im Schnitt bei 4,29 %. Real, ohne Staking, sind es 1,07 %. Pro Karte werden im Schnitt nur 34 % des beworbenen Cashbacks gezahlt. Jede zweite Karte zahlt gar keinen Basis-Cashback. Der größte Abstand: Bleap, 20 % beworben, 1 % real.
+Alle Zahlen sind handgeprüft, nach Land aufgeschlüsselt, mit offener Methodik: https://topcryptocards.eu/etudes/krypto-karten-2026
+Gern liefere ich die vollständigen Daten pro Karte, Zahlen für den DACH-Raum oder ein Zitat.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -2738,6 +3617,21 @@
       <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="7" t="inlineStr"/>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Datenstudie: Krypto-Karten zahlen nur 34 % des versprochenen Cashbacks</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>Hallo Redaktion,
+ein Verbraucherthema mit eigenen Daten.
+Wir haben 93 in Europa verfügbare Krypto-Karten ausgewertet. Der beworbene Cashback liegt im Schnitt bei 4,29 %. Real, ohne Staking, sind es 1,07 %. Pro Karte werden im Schnitt nur 34 % des beworbenen Cashbacks gezahlt. Jede zweite Karte zahlt gar keinen Basis-Cashback. Der größte Abstand: Bleap, 20 % beworben, 1 % real.
+Alle Zahlen sind handgeprüft, nach Land aufgeschlüsselt, mit offener Methodik: https://topcryptocards.eu/etudes/krypto-karten-2026
+Gern liefere ich die vollständigen Daten pro Karte, Zahlen für den DACH-Raum oder ein Zitat.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2783,6 +3677,21 @@
       <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Estudio con datos: las tarjetas cripto pagan solo el 34 % del cashback que prometen</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Hola,
+Un ángulo de consumo con datos propios.
+Hemos analizado 95 tarjetas cripto disponibles en Europa. El cashback anunciado es del 4,29 % de media. El real, sin staking, baja al 1,07 %. Por tarjeta, de media solo se paga el 34 % del cashback anunciado. Una de cada dos tarjetas no da cashback base. La mayor diferencia es Bleap, 20 % anunciado frente a 1 % real.
+Cada cifra está verificada a mano, desglosada por país y con metodología abierta: https://topcryptocards.eu/etudes/tarjetas-cripto-2026
+Puedo facilitar los datos completos por tarjeta, cifras del mercado español o una cita.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2828,6 +3737,21 @@
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="7" t="inlineStr"/>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Estudio con datos: las tarjetas cripto pagan solo el 34 % del cashback que prometen</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>Hola,
+Un ángulo de consumo con datos propios.
+Hemos analizado 95 tarjetas cripto disponibles en Europa. El cashback anunciado es del 4,29 % de media. El real, sin staking, baja al 1,07 %. Por tarjeta, de media solo se paga el 34 % del cashback anunciado. Una de cada dos tarjetas no da cashback base. La mayor diferencia es Bleap, 20 % anunciado frente a 1 % real.
+Cada cifra está verificada a mano, desglosada por país y con metodología abierta: https://topcryptocards.eu/etudes/tarjetas-cripto-2026
+Puedo facilitar los datos completos por tarjeta, cifras del mercado español o una cita.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2873,6 +3797,21 @@
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Estudio con datos: las tarjetas cripto pagan solo el 34 % del cashback que prometen</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Hola,
+Un ángulo de consumo con datos propios.
+Hemos analizado 95 tarjetas cripto disponibles en Europa. El cashback anunciado es del 4,29 % de media. El real, sin staking, baja al 1,07 %. Por tarjeta, de media solo se paga el 34 % del cashback anunciado. Una de cada dos tarjetas no da cashback base. La mayor diferencia es Bleap, 20 % anunciado frente a 1 % real.
+Cada cifra está verificada a mano, desglosada por país y con metodología abierta: https://topcryptocards.eu/etudes/tarjetas-cripto-2026
+Puedo facilitar los datos completos por tarjeta, cifras del mercado español o una cita.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2902,7 +3841,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>via articles + LinkedIn</t>
+          <t>page contact rédaction du média</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -2918,6 +3857,21 @@
       <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Estudio con datos: las tarjetas cripto pagan solo el 34 % del cashback que prometen</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>Hola,
+Un ángulo de consumo con datos propios.
+Hemos analizado 95 tarjetas cripto disponibles en Europa. El cashback anunciado es del 4,29 % de media. El real, sin staking, baja al 1,07 %. Por tarjeta, de media solo se paga el 34 % del cashback anunciado. Una de cada dos tarjetas no da cashback base. La mayor diferencia es Bleap, 20 % anunciado frente a 1 % real.
+Cada cifra está verificada a mano, desglosada por país y con metodología abierta: https://topcryptocards.eu/etudes/tarjetas-cripto-2026
+Puedo facilitar los datos completos por tarjeta, cifras del mercado español o una cita.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2947,7 +3901,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>cryptonomist.ch (contatti) · LinkedIn</t>
+          <t>cryptonomist.ch (contatti)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -2963,6 +3917,21 @@
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Studio con dati: le carte crypto pagano solo il 34 % del cashback promesso</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Salve,
+Un taglio consumer con dati originali.
+Abbiamo analizzato 95 carte crypto disponibili in Europa. Il cashback pubblicizzato è in media del 4,29 %. Quello reale, senza staking, scende allo 1,07 %. Per carta, in media viene versato solo il 34 % del cashback pubblicizzato. Una carta su due non dà alcun cashback base. Il divario più ampio è Bleap, 20 % pubblicizzato contro 1 % reale.
+Ogni dato è verificato a mano, suddiviso per paese, con metodologia aperta: https://topcryptocards.eu/etudes/carte-crypto-2026
+Posso fornire i dati completi per carta, i numeri del mercato italiano o una dichiarazione.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -3008,6 +3977,21 @@
       <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr"/>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>Studio con dati: le carte crypto pagano solo il 34 % del cashback promesso</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>Salve,
+Un taglio consumer con dati originali.
+Abbiamo analizzato 95 carte crypto disponibili in Europa. Il cashback pubblicizzato è in media del 4,29 %. Quello reale, senza staking, scende allo 1,07 %. Per carta, in media viene versato solo il 34 % del cashback pubblicizzato. Una carta su due non dà alcun cashback base. Il divario più ampio è Bleap, 20 % pubblicizzato contro 1 % reale.
+Ogni dato è verificato a mano, suddiviso per paese, con metodologia aperta: https://topcryptocards.eu/etudes/carte-crypto-2026
+Posso fornire i dati completi per carta, i numeri del mercato italiano o una dichiarazione.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -3053,6 +4037,21 @@
       <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="6" t="inlineStr"/>
       <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>Studio con dati: le carte crypto pagano solo il 34 % del cashback promesso</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>Salve,
+Un taglio consumer con dati originali.
+Abbiamo analizzato 95 carte crypto disponibili in Europa. Il cashback pubblicizzato è in media del 4,29 %. Quello reale, senza staking, scende allo 1,07 %. Per carta, in media viene versato solo il 34 % del cashback pubblicizzato. Una carta su due non dà alcun cashback base. Il divario più ampio è Bleap, 20 % pubblicizzato contro 1 % reale.
+Ogni dato è verificato a mano, suddiviso per paese, con metodologia aperta: https://topcryptocards.eu/etudes/carte-crypto-2026
+Posso fornire i dati completi per carta, i numeri del mercato italiano o una dichiarazione.
+Thomas, TopCryptoCards</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K11"/>

</xml_diff>